<commit_message>
data: update 고객사현황.xlsx for 2026-08-28
</commit_message>
<xml_diff>
--- a/docs/dashboard/data/고객사현황.xlsx
+++ b/docs/dashboard/data/고객사현황.xlsx
@@ -98,7 +98,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="15.0" customWidth="true"/>
@@ -174,37 +174,37 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-004</t>
+          <t>GG-M-26-012</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>(주)대성티엠씨</t>
+          <t>디지트론</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>경기도 성남시 수정구</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>6068641818</t>
+          <t>1298603001</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>노윤재</t>
+          <t>이종국</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>유신재</t>
+          <t>정재종</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>010-5307-6284</t>
+          <t>010-4511-4977</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -217,7 +217,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>이정수</t>
+          <t>정태화</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -229,41 +229,41 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>JB-M-26-001</t>
+          <t>GN-S-26-001</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>오씨아이파워주식회사</t>
+          <t>현대건설(주)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>전북특별자치도 군산시</t>
+          <t>경상북도 울진군</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>1048644532</t>
+          <t>1018116293</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>김성엽</t>
+          <t>이한우</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>추혜빈</t>
+          <t>김태호</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>010-9193-6015</t>
+          <t>010-4027-1418</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -272,7 +272,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>이승봉</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -284,37 +284,37 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CN-A-26-002</t>
+          <t>GN-M-26-004</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>세일전장 주식회사</t>
+          <t>(주)대성티엠씨</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>충청남도 홍성군</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2218802452</t>
+          <t>6068641818</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>고승근</t>
+          <t>노윤재</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>홍유성</t>
+          <t>유신재</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>010-4054-0831</t>
+          <t>010-5307-6284</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -327,49 +327,49 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>이정수</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-004</t>
+          <t>JB-M-26-001</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>(주)동광보일러</t>
+          <t>오씨아이파워주식회사</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>충청남도 아산시</t>
+          <t>전북특별자치도 군산시</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>1408121883</t>
+          <t>1048644532</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>박정연</t>
+          <t>김성엽</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>김용휘</t>
+          <t>추혜빈</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>010-9731-5222</t>
+          <t>010-9193-6015</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -387,44 +387,44 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-003</t>
+          <t>CN-A-26-002</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>(주)센추리 아산공장</t>
+          <t>세일전장 주식회사</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>충청남도 아산시</t>
+          <t>충청남도 홍성군</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>3128545076</t>
+          <t>2218802452</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>백현수,최진민</t>
+          <t>고승근</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>허민영</t>
+          <t>홍유성</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>010-8484-3476</t>
+          <t>010-4054-0831</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -449,12 +449,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-002</t>
+          <t>CN-M-26-004</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에이치엔에프</t>
+          <t>(주)동광보일러</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -464,22 +464,22 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>7398801954</t>
+          <t>1408121883</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>이형욱</t>
+          <t>박정연</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>조수형</t>
+          <t>김용휘</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>010-2310-3404</t>
+          <t>010-9731-5222</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -504,37 +504,37 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-005</t>
+          <t>CN-M-26-003</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
+          <t>(주)센추리 아산공장</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>경기도 오산시</t>
+          <t>충청남도 아산시</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>8858800321</t>
+          <t>3128545076</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>엄월용</t>
+          <t>백현수,최진민</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>사금석</t>
+          <t>허민영</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>010-8832-0250</t>
+          <t>010-8484-3476</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -559,37 +559,37 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-004</t>
+          <t>CN-M-26-002</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
+          <t>주식회사 에이치엔에프</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>경기도 화성시 동탄구</t>
+          <t>충청남도 아산시</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>7888101296</t>
+          <t>7398801954</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>XIANGXIFEI</t>
+          <t>이형욱</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>박은범</t>
+          <t>조수형</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>010-9335-4934</t>
+          <t>010-2310-3404</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -614,37 +614,37 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>SE-M-26-007</t>
+          <t>GG-E-26-005</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>주식회사 엑소퍼트(EXoPERT CORPORATION)</t>
+          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 동대문구</t>
+          <t>경기도 오산시</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>5318701197</t>
+          <t>8858800321</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>최연호</t>
+          <t>엄월용</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>전소희</t>
+          <t>사금석</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>010-5228-4793</t>
+          <t>010-8832-0250</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -657,7 +657,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -669,37 +669,37 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GG-F-26-001</t>
+          <t>GG-E-26-004</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>태광푸드(주)</t>
+          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>경기도 파주시</t>
+          <t>경기도 화성시 동탄구</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>1508701192</t>
+          <t>7888101296</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>김성재</t>
+          <t>XIANGXIFEI</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>김영은</t>
+          <t>박은범</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>010-9559-7211</t>
+          <t>010-9335-4934</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -712,7 +712,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -724,37 +724,37 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SE-S-26-002</t>
+          <t>SE-M-26-007</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>노을그린에너지 주식회사</t>
+          <t>주식회사 엑소퍼트(EXoPERT CORPORATION)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 마포구</t>
+          <t>서울특별시 동대문구</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>1058807174</t>
+          <t>5318701197</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>고창석</t>
+          <t>최연호</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>정진호</t>
+          <t>전소희</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>010-9931-3764</t>
+          <t>010-5228-4793</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -779,37 +779,37 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>GG-S-26-004</t>
+          <t>GG-F-26-001</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>김포골드라인에스알에스 주식회사</t>
+          <t>태광푸드(주)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>경기도 파주시</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>6258803309</t>
+          <t>1508701192</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>이수호</t>
+          <t>김성재</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>박성주</t>
+          <t>김영은</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>010-7195-7524</t>
+          <t>010-9559-7211</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -834,37 +834,37 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-011</t>
+          <t>SE-S-26-002</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>주식회사 싱크홀</t>
+          <t>노을그린에너지 주식회사</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>서울특별시 마포구</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>6798502456</t>
+          <t>1058807174</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>정대성</t>
+          <t>고창석</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>신현석</t>
+          <t>정진호</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>010-9760-0559</t>
+          <t>010-9931-3764</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -889,37 +889,37 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-010</t>
+          <t>GG-S-26-004</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>대동도어주식회사</t>
+          <t>김포골드라인에스알에스 주식회사</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 연수구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>1348173163</t>
+          <t>6258803309</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>송학성</t>
+          <t>이수호</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>조예지</t>
+          <t>박성주</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>010-9278-6791</t>
+          <t>010-7195-7524</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -944,37 +944,37 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>GG-S-26-003</t>
+          <t>GG-M-26-011</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>지티엑스에이운영(주)</t>
+          <t>주식회사 싱크홀</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>경기도 고양시 덕양구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>8738702917</t>
+          <t>6798502456</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>서길호</t>
+          <t>정대성</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>이성호</t>
+          <t>신현석</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>010-9093-0316</t>
+          <t>010-9760-0559</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -999,37 +999,37 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-009</t>
+          <t>GG-M-26-010</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>영상폴리텍</t>
+          <t>대동도어주식회사</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>인천광역시 연수구</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>1312660786</t>
+          <t>1348173163</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>전영식</t>
+          <t>송학성</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>오세준</t>
+          <t>조예지</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>010-3940-5634</t>
+          <t>010-9278-6791</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -1054,37 +1054,37 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>GW-S-26-001</t>
+          <t>GG-S-26-003</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>주식회사 파라타항공</t>
+          <t>지티엑스에이운영(주)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>강원특별자치도 양양군</t>
+          <t>경기도 고양시 덕양구</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>7108100367</t>
+          <t>8738702917</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>윤철민</t>
+          <t>서길호</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>변태웅</t>
+          <t>이성호</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>010-2882-5159</t>
+          <t>010-9093-0316</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -1109,37 +1109,37 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>GG-B-26-002</t>
+          <t>GG-M-26-009</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>대한약품공업(주)반월공장</t>
+          <t>영상폴리텍</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>1348500111</t>
+          <t>1312660786</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>이승영</t>
+          <t>전영식</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>이성원</t>
+          <t>오세준</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>010-4188-2847</t>
+          <t>010-3940-5634</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
@@ -1164,37 +1164,37 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>GG-A-26-002</t>
+          <t>GG-B-26-002</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>주식회사 대솔오시스</t>
+          <t>대한약품공업(주)반월공장</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 안산시 단원구</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>1398115533</t>
+          <t>1348500111</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>권민호</t>
+          <t>이승영</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>장지은</t>
+          <t>이성원</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>010-7141-6474</t>
+          <t>010-4188-2847</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
@@ -1219,37 +1219,37 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-008</t>
+          <t>GG-A-26-002</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>케이젯정밀 (주) 펌프공장</t>
+          <t>주식회사 대솔오시스</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>1348501217</t>
+          <t>1398115533</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>이한성</t>
+          <t>권민호</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>왕대영</t>
+          <t>장지은</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>010-8882-9381</t>
+          <t>010-7141-6474</t>
         </is>
       </c>
       <c r="H21" s="2" t="n">
@@ -1274,37 +1274,37 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-007</t>
+          <t>GG-A-26-001</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>케이젯정밀 (주) 밸브공장</t>
+          <t>(주) 대한솔루션</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>1348555479</t>
+          <t>1398100699</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>이한성</t>
+          <t>권회현, 오문석, 권충호</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>이샘솔</t>
+          <t>윤종혁</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>010-4105-0907</t>
+          <t>010-9252-5623</t>
         </is>
       </c>
       <c r="H22" s="2" t="n">
@@ -1329,12 +1329,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>GG-A-26-001</t>
+          <t>GG-M-26-006</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>(주) 대한솔루션</t>
+          <t>(주)오성기전</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1344,22 +1344,22 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>1398100699</t>
+          <t>1318629038</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>권회현, 오문석, 권충호</t>
+          <t>장순보</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>윤종혁</t>
+          <t>이미래</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>010-9252-5623</t>
+          <t>010-2513-4454</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
@@ -1384,41 +1384,41 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-006</t>
+          <t>GG-M-26-005</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>(주)오성기전</t>
+          <t>(주)윤성에프앤씨</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 안성시</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>1318629038</t>
+          <t>1348150350</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>장순보</t>
+          <t>박치영</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>이미래</t>
+          <t>윤성현</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>010-2513-4454</t>
+          <t>010-9914-7989</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>0.0</v>
+        <v>288.0</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -1439,41 +1439,41 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-005</t>
+          <t>GG-M-26-004</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>(주)윤성에프앤씨</t>
+          <t>(주)백콤</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>경기도 안성시</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>1348150350</t>
+          <t>1308628716</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>박치영</t>
+          <t>이석원</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>윤성현</t>
+          <t>서범석</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>010-9914-7989</t>
+          <t>010-5055-4994</t>
         </is>
       </c>
       <c r="H25" s="2" t="n">
-        <v>0.0</v>
+        <v>47.0</v>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
@@ -1482,53 +1482,53 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-004</t>
+          <t>GG-M-26-003</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>(주)백콤</t>
+          <t>한국미쓰비시엘리베이터(주)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>인천광역시 연수구</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>1308628716</t>
+          <t>1378514007</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>이석원</t>
+          <t>김성빈</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>서범석</t>
+          <t>장연욱</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>010-5055-4994</t>
+          <t>010-3976-0627</t>
         </is>
       </c>
       <c r="H26" s="2" t="n">
-        <v>47.0</v>
+        <v>209.0</v>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
@@ -1549,92 +1549,92 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-003</t>
+          <t>GG-S-26-002</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>한국미쓰비시엘리베이터(주)</t>
+          <t>주식회사 웨이투웨이</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 연수구</t>
+          <t>경기 시흥시</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>1378514007</t>
+          <t>1408181673</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>김성빈</t>
+          <t>민금기</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>장연욱</t>
+          <t>김미선</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>010-3976-0627</t>
+          <t>010-9301-4564</t>
         </is>
       </c>
       <c r="H27" s="2" t="n">
-        <v>209.0</v>
+        <v>0.0</v>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>정상</t>
+          <t>비활성</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>최승혜</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>GG-S-26-002</t>
+          <t>GG-M-26-002</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>주식회사 웨이투웨이</t>
+          <t>비카코리아 주식회사</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>경기 시흥시</t>
+          <t>경기도 오산시</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>1408181673</t>
+          <t>6108128707</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>민금기</t>
+          <t>이덕우</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>김미선</t>
+          <t>이진형</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>010-9301-4564</t>
+          <t>010-4026-3019</t>
         </is>
       </c>
       <c r="H28" s="2" t="n">
@@ -1642,58 +1642,58 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>비활성</t>
+          <t>정상</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>최승혜</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-002</t>
+          <t>CN-E-26-001</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>비카코리아 주식회사</t>
+          <t>(주)디바이스</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>경기도 오산시</t>
+          <t>충청남도 천안시 서북구</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>6108128707</t>
+          <t>3128157991</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>이덕우</t>
+          <t>최봉진, 방인호</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>이진형</t>
+          <t>김용호</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>010-4026-3019</t>
+          <t>010-3474-3716</t>
         </is>
       </c>
       <c r="H29" s="2" t="n">
-        <v>0.0</v>
+        <v>70.0</v>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
@@ -1714,41 +1714,41 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>CN-E-26-001</t>
+          <t>GG-E-26-003</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>(주)디바이스</t>
+          <t>(주)지에프에스</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>충청남도 천안시 서북구</t>
+          <t>경기도 의정부시</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>3128157991</t>
+          <t>1278107419</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>최봉진, 방인호</t>
+          <t>김태호,김현식</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>김용호</t>
+          <t>임승현</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>010-3474-3716</t>
+          <t>010-9516-5508</t>
         </is>
       </c>
       <c r="H30" s="2" t="n">
-        <v>70.0</v>
+        <v>0.0</v>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
@@ -1757,53 +1757,53 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>김경훈</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-003</t>
+          <t>GB-M-26-001</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>(주)지에프에스</t>
+          <t>(주)케이피씨엠</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>경기도 의정부시</t>
+          <t>경상북도 경산시</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>1278107419</t>
+          <t>5158140973</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>김태호,김현식</t>
+          <t>안장홍</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>임승현</t>
+          <t>이예슬</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>010-9516-5508</t>
+          <t>010-9721-4885</t>
         </is>
       </c>
       <c r="H31" s="2" t="n">
-        <v>0.0</v>
+        <v>188.0</v>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>김경훈</t>
+          <t>한규범</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -1824,41 +1824,41 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>GB-M-26-001</t>
+          <t>SE-E-26-002</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>(주)케이피씨엠</t>
+          <t>(주)경인기술</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>경상북도 경산시</t>
+          <t>서울특별시 영등포구</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>5158140973</t>
+          <t>1138156416</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>안장홍</t>
+          <t>정진흥</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>이예슬</t>
+          <t>임성종</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>010-9721-4885</t>
+          <t>010-2905-7307</t>
         </is>
       </c>
       <c r="H32" s="2" t="n">
-        <v>188.0</v>
+        <v>0.0</v>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
@@ -1867,49 +1867,49 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>한규범</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>SE-E-26-002</t>
+          <t>GG-E-26-002</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>(주)경인기술</t>
+          <t>(주)코리아하이텍</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 영등포구</t>
+          <t>경기도 안산시 단원구</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>1138156416</t>
+          <t>1348106311</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>정진흥</t>
+          <t>여승훈,오석철</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>임성종</t>
+          <t>박진우</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>010-2905-7307</t>
+          <t>010-6377-6757</t>
         </is>
       </c>
       <c r="H33" s="2" t="n">
@@ -1934,41 +1934,41 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-002</t>
+          <t>SE-S-26-001</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>(주)코리아하이텍</t>
+          <t>에브제트아시아(주)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>서울특별시 강서구</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>1348106311</t>
+          <t>1208731282</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>여승훈,오석철</t>
+          <t>조욱상</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>박진우</t>
+          <t>전승헌</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>010-6377-6757</t>
+          <t>010-8833-0349</t>
         </is>
       </c>
       <c r="H34" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
@@ -1989,41 +1989,41 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>SE-S-26-001</t>
+          <t>GN-M-26-003</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>에브제트아시아(주)</t>
+          <t>디엔엠항공</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 강서구</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>1208731282</t>
+          <t>6131783159</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>조욱상</t>
+          <t>황태부</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>전승헌</t>
+          <t>김미희</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>010-8833-0349</t>
+          <t>010-8131-0888</t>
         </is>
       </c>
       <c r="H35" s="2" t="n">
-        <v>1.0</v>
+        <v>452.0</v>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>이정수</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -2044,41 +2044,41 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-003</t>
+          <t>GG-M-26-001</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>디엔엠항공</t>
+          <t>씨트론(주)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>인천광역시 계양구</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>6131783159</t>
+          <t>1228159023</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>황태부</t>
+          <t>정태화</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>김미희</t>
+          <t>양혜원</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>010-8131-0888</t>
+          <t>010-2770-7226</t>
         </is>
       </c>
       <c r="H36" s="2" t="n">
-        <v>452.0</v>
+        <v>0.0</v>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>이정수</t>
+          <t>이승건</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -2099,37 +2099,37 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-001</t>
+          <t>GG-B-26-001</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>씨트론(주)</t>
+          <t>(주)알피바이오</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 계양구</t>
+          <t>경기도 화성시 만세구</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>1228159023</t>
+          <t>7758501361</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>정태화</t>
+          <t>윤재훈</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>양혜원</t>
+          <t>노승우</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>010-2770-7226</t>
+          <t>010-4899-3983</t>
         </is>
       </c>
       <c r="H37" s="2" t="n">
@@ -2154,41 +2154,41 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>GG-B-26-001</t>
+          <t>SE-B-26-001</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>(주)알피바이오</t>
+          <t>주식회사 코젠바이오텍</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>경기도 화성시 만세구</t>
+          <t>서울특별시 금천구</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>7758501361</t>
+          <t>1018156320</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>윤재훈</t>
+          <t>남용석, 남주현</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>노승우</t>
+          <t>정지만</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>010-4899-3983</t>
+          <t>010-5348-2308</t>
         </is>
       </c>
       <c r="H38" s="2" t="n">
-        <v>0.0</v>
+        <v>45.0</v>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>이승건</t>
+          <t>정경훈</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -2209,41 +2209,41 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>SE-B-26-001</t>
+          <t>GG-S-26-001</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>주식회사 코젠바이오텍</t>
+          <t>(주)에어로피스</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 금천구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>1018156320</t>
+          <t>1378604165</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>남용석, 남주현</t>
+          <t>송인성</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>정지만</t>
+          <t>염요찬</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>010-5348-2308</t>
+          <t>010-8803-5930</t>
         </is>
       </c>
       <c r="H39" s="2" t="n">
-        <v>45.0</v>
+        <v>237.0</v>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>정경훈</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
@@ -2264,41 +2264,41 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>GG-S-26-001</t>
+          <t>SE-M-26-006</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>(주)에어로피스</t>
+          <t>주식회사 덱스레보</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>서울 금천구</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>1378604165</t>
+          <t>1198678150</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>송인성</t>
+          <t>유재원</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>염요찬</t>
+          <t>이득훈</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>010-8803-5930</t>
+          <t>010-4119-7124</t>
         </is>
       </c>
       <c r="H40" s="2" t="n">
-        <v>237.0</v>
+        <v>10.0</v>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>정경훈</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -2319,41 +2319,41 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>SE-M-26-006</t>
+          <t>GN-M-26-002</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>주식회사 덱스레보</t>
+          <t>주식회사 카프마이크로</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>서울 금천구</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>1198678150</t>
+          <t>3148613655</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>유재원</t>
+          <t>이인권</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>이득훈</t>
+          <t>박준영</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>010-4119-7124</t>
+          <t>010-9305-1034</t>
         </is>
       </c>
       <c r="H41" s="2" t="n">
-        <v>10.0</v>
+        <v>60.0</v>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
@@ -2362,53 +2362,53 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>정경훈</t>
+          <t>이정수</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-002</t>
+          <t>CN-M-26-001</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>주식회사 카프마이크로</t>
+          <t>연합정밀(주)</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>충남 천안시 동남구</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>3148613655</t>
+          <t>3128109219</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>이인권</t>
+          <t>김은주</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>박준영</t>
+          <t>하상우</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>010-9305-1034</t>
+          <t>010-2942-3411</t>
         </is>
       </c>
       <c r="H42" s="2" t="n">
-        <v>60.0</v>
+        <v>1827.0</v>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>이정수</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -2429,41 +2429,41 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-001</t>
+          <t>SE-E-26-001</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>연합정밀(주)</t>
+          <t>(주)우리기술</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>충남 천안시 동남구</t>
+          <t>서울 마포구</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>3128109219</t>
+          <t>1128138619</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>김은주</t>
+          <t>노갑선</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>하상우</t>
+          <t>이원근</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>010-2942-3411</t>
+          <t>010-9792-8173</t>
         </is>
       </c>
       <c r="H43" s="2" t="n">
-        <v>1827.0</v>
+        <v>84.0</v>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
@@ -2472,53 +2472,53 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>SE-E-26-001</t>
+          <t>GN-M-26-001</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>(주)우리기술</t>
+          <t>(주)신화프리텍</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>서울 마포구</t>
+          <t>경남 창원시 성산구</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>1128138619</t>
+          <t>6088151660</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>노갑선</t>
+          <t>배진기</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>이원근</t>
+          <t>최문정</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>010-9792-8173</t>
+          <t>010-8669-1533</t>
         </is>
       </c>
       <c r="H44" s="2" t="n">
-        <v>84.0</v>
+        <v>1070.0</v>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>송민규</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -2539,41 +2539,41 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-001</t>
+          <t>CB-A-26-001</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>(주)신화프리텍</t>
+          <t>(주)한국기능공사</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>경남 창원시 성산구</t>
+          <t>충북 음성군</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>6088151660</t>
+          <t>1258112293</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>배진기</t>
+          <t>김성국, 김성만</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>최문정</t>
+          <t>하갑봉</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>010-8669-1533</t>
+          <t>010-5655-3719</t>
         </is>
       </c>
       <c r="H45" s="2" t="n">
-        <v>1070.0</v>
+        <v>614.0</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>송민규</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -2594,41 +2594,41 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>CB-A-26-001</t>
+          <t>GG-E-26-001</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>(주)한국기능공사</t>
+          <t>(주)휴니드테크놀러지스</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>충북 음성군</t>
+          <t>인천 연수구</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>1258112293</t>
+          <t>1238106174</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>김성국, 김성만</t>
+          <t>이철승(공동대표),김영호(공동대표)</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>하갑봉</t>
+          <t>신원범</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>010-5655-3719</t>
+          <t>010-8543-4717</t>
         </is>
       </c>
       <c r="H46" s="2" t="n">
-        <v>614.0</v>
+        <v>916.0</v>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
@@ -2637,53 +2637,53 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-001</t>
+          <t>CN-A-26-001</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>(주)휴니드테크놀러지스</t>
+          <t>(주)서연이화 아산공장</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>인천 연수구</t>
+          <t>충남 아산시</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>1238106174</t>
+          <t>3128564374</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>이철승(공동대표),김영호(공동대표)</t>
+          <t>강용석</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>신원범</t>
+          <t>류제형</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>010-8543-4717</t>
+          <t>010-8210-1082</t>
         </is>
       </c>
       <c r="H47" s="2" t="n">
-        <v>916.0</v>
+        <v>84.0</v>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -2704,108 +2704,53 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>CN-A-26-001</t>
+          <t>SE-M-26-005</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>(주)서연이화 아산공장</t>
+          <t>코리아인스트루먼트(주)</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>충남 아산시</t>
+          <t>서울 구로구</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>3128564374</t>
+          <t>1018145861</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>강용석</t>
+          <t>최선구</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>류제형</t>
+          <t>KIC관리자</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>010-8210-1082</t>
+          <t>010-0000-0000</t>
         </is>
       </c>
       <c r="H48" s="2" t="n">
-        <v>84.0</v>
+        <v>0.0</v>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>정상</t>
+          <t>비활성</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>KIC관리자</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>SE-M-26-005</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>코리아인스트루먼트(주)</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>서울 구로구</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>1018145861</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>최선구</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>KIC관리자</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="inlineStr">
-        <is>
-          <t>010-0000-0000</t>
-        </is>
-      </c>
-      <c r="H49" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="I49" s="2" t="inlineStr">
-        <is>
-          <t>비활성</t>
-        </is>
-      </c>
-      <c r="J49" s="2" t="inlineStr">
-        <is>
-          <t>KIC관리자</t>
-        </is>
-      </c>
-      <c r="K49" s="2" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>

</xml_diff>

<commit_message>
data: update 고객사현황.xlsx for 2026-09-04
</commit_message>
<xml_diff>
--- a/docs/dashboard/data/고객사현황.xlsx
+++ b/docs/dashboard/data/고객사현황.xlsx
@@ -98,7 +98,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="15.0" customWidth="true"/>
@@ -174,41 +174,41 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-012</t>
+          <t>GN-M-26-005</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>디지트론</t>
+          <t>하이에어코리아(주)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>경기도 성남시 수정구</t>
+          <t>경상남도 김해시</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>1298603001</t>
+          <t>6038110081</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>이종국</t>
+          <t>김근배,김태홍</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>정재종</t>
+          <t>황동환</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>010-4511-4977</t>
+          <t>010-4556-5585</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0.0</v>
+        <v>11.0</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -217,53 +217,53 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>정태화</t>
+          <t>한규범</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>GN-S-26-001</t>
+          <t>CB-A-26-002</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>현대건설(주)</t>
+          <t>보그워너충주 유한책임회사</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>경상북도 울진군</t>
+          <t>충청북도 충주시</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>1018116293</t>
+          <t>3038108176</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>이한우</t>
+          <t>박귀선</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>김태호</t>
+          <t>김혜진</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>010-4027-1418</t>
+          <t>010-8668-5752</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -272,53 +272,53 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>이승봉</t>
+          <t>박민경</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-004</t>
+          <t>GG-M-26-012</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>(주)대성티엠씨</t>
+          <t>디지트론</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>경기도 성남시 수정구</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>6068641818</t>
+          <t>1298603001</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>노윤재</t>
+          <t>이종국</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>유신재</t>
+          <t>정재종</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>010-5307-6284</t>
+          <t>010-4511-4977</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -327,7 +327,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>이정수</t>
+          <t>정태화</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -339,41 +339,41 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>JB-M-26-001</t>
+          <t>GN-S-26-001</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>오씨아이파워주식회사</t>
+          <t>현대건설(주)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>전북특별자치도 군산시</t>
+          <t>경상북도 울진군</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>1048644532</t>
+          <t>1018116293</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>김성엽</t>
+          <t>이한우</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>추혜빈</t>
+          <t>김태호</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>010-9193-6015</t>
+          <t>010-4027-1418</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -382,7 +382,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>이승봉</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -394,37 +394,37 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>CN-A-26-002</t>
+          <t>GN-M-26-004</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>세일전장 주식회사</t>
+          <t>(주)대성티엠씨</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>충청남도 홍성군</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2218802452</t>
+          <t>6068641818</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>고승근</t>
+          <t>노윤재</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>홍유성</t>
+          <t>유신재</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>010-4054-0831</t>
+          <t>010-5307-6284</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -437,49 +437,49 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>이정수</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-004</t>
+          <t>JB-M-26-001</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>(주)동광보일러</t>
+          <t>오씨아이파워주식회사</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>충청남도 아산시</t>
+          <t>전북특별자치도 군산시</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>1408121883</t>
+          <t>1048644532</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>박정연</t>
+          <t>김성엽</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>김용휘</t>
+          <t>추혜빈</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>010-9731-5222</t>
+          <t>010-9193-6015</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -497,44 +497,44 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-003</t>
+          <t>CN-A-26-002</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>(주)센추리 아산공장</t>
+          <t>세일전장 주식회사</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>충청남도 아산시</t>
+          <t>충청남도 홍성군</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>3128545076</t>
+          <t>2218802452</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>백현수,최진민</t>
+          <t>고승근</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>허민영</t>
+          <t>홍유성</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>010-8484-3476</t>
+          <t>010-4054-0831</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -559,12 +559,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-002</t>
+          <t>CN-M-26-004</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에이치엔에프</t>
+          <t>(주)동광보일러</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -574,22 +574,22 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>7398801954</t>
+          <t>1408121883</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>이형욱</t>
+          <t>박정연</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>조수형</t>
+          <t>김용휘</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>010-2310-3404</t>
+          <t>010-9731-5222</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -614,41 +614,41 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-005</t>
+          <t>CN-M-26-003</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
+          <t>(주)센추리 아산공장</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>경기도 오산시</t>
+          <t>충청남도 아산시</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>8858800321</t>
+          <t>3128545076</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>엄월용</t>
+          <t>백현수,최진민</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>사금석</t>
+          <t>허민영</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>010-8832-0250</t>
+          <t>010-8484-3476</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0.0</v>
+        <v>293.0</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -669,37 +669,37 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-004</t>
+          <t>CN-M-26-002</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
+          <t>주식회사 에이치엔에프</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>경기도 화성시 동탄구</t>
+          <t>충청남도 아산시</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>7888101296</t>
+          <t>7398801954</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>XIANGXIFEI</t>
+          <t>이형욱</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>박은범</t>
+          <t>조수형</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>010-9335-4934</t>
+          <t>010-2310-3404</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -724,37 +724,37 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SE-M-26-007</t>
+          <t>GG-E-26-005</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>주식회사 엑소퍼트(EXoPERT CORPORATION)</t>
+          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 동대문구</t>
+          <t>경기도 오산시</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>5318701197</t>
+          <t>8858800321</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>최연호</t>
+          <t>엄월용</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>전소희</t>
+          <t>사금석</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>010-5228-4793</t>
+          <t>010-8832-0250</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -767,7 +767,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -779,37 +779,37 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>GG-F-26-001</t>
+          <t>GG-E-26-004</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>태광푸드(주)</t>
+          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>경기도 파주시</t>
+          <t>경기도 화성시 동탄구</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>1508701192</t>
+          <t>7888101296</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>김성재</t>
+          <t>XIANGXIFEI</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>김영은</t>
+          <t>박은범</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>010-9559-7211</t>
+          <t>010-9335-4934</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -822,7 +822,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -834,37 +834,37 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>SE-S-26-002</t>
+          <t>SE-M-26-007</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>노을그린에너지 주식회사</t>
+          <t>주식회사 엑소퍼트(EXoPERT CORPORATION)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 마포구</t>
+          <t>서울특별시 동대문구</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>1058807174</t>
+          <t>5318701197</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>고창석</t>
+          <t>최연호</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>정진호</t>
+          <t>전소희</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>010-9931-3764</t>
+          <t>010-5228-4793</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -889,37 +889,37 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>GG-S-26-004</t>
+          <t>GG-F-26-001</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>김포골드라인에스알에스 주식회사</t>
+          <t>태광푸드(주)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>경기도 파주시</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>6258803309</t>
+          <t>1508701192</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>이수호</t>
+          <t>김성재</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>박성주</t>
+          <t>김영은</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>010-7195-7524</t>
+          <t>010-9559-7211</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -944,37 +944,37 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-011</t>
+          <t>SE-S-26-002</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>주식회사 싱크홀</t>
+          <t>노을그린에너지 주식회사</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>서울특별시 마포구</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>6798502456</t>
+          <t>1058807174</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>정대성</t>
+          <t>고창석</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>신현석</t>
+          <t>정진호</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>010-9760-0559</t>
+          <t>010-9931-3764</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -999,37 +999,37 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-010</t>
+          <t>GG-S-26-004</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>대동도어주식회사</t>
+          <t>김포골드라인에스알에스 주식회사</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 연수구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>1348173163</t>
+          <t>6258803309</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>송학성</t>
+          <t>이수호</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>조예지</t>
+          <t>박성주</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>010-9278-6791</t>
+          <t>010-7195-7524</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -1054,37 +1054,37 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>GG-S-26-003</t>
+          <t>GG-M-26-011</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>지티엑스에이운영(주)</t>
+          <t>주식회사 싱크홀</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>경기도 고양시 덕양구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>8738702917</t>
+          <t>6798502456</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>서길호</t>
+          <t>정대성</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>이성호</t>
+          <t>신현석</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>010-9093-0316</t>
+          <t>010-9760-0559</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -1109,37 +1109,37 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-009</t>
+          <t>GG-S-26-003</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>영상폴리텍</t>
+          <t>지티엑스에이운영(주)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 고양시 덕양구</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>1312660786</t>
+          <t>8738702917</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>전영식</t>
+          <t>서길호</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>오세준</t>
+          <t>이성호</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>010-3940-5634</t>
+          <t>010-9093-0316</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
@@ -1164,37 +1164,37 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>GG-B-26-002</t>
+          <t>GG-M-26-009</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>대한약품공업(주)반월공장</t>
+          <t>영상폴리텍</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>1348500111</t>
+          <t>1312660786</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>이승영</t>
+          <t>전영식</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>이성원</t>
+          <t>오세준</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>010-4188-2847</t>
+          <t>010-3940-5634</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
@@ -1219,41 +1219,41 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>GG-A-26-002</t>
+          <t>GG-B-26-002</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>주식회사 대솔오시스</t>
+          <t>대한약품공업(주)반월공장</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 안산시 단원구</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>1398115533</t>
+          <t>1348500111</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>권민호</t>
+          <t>이승영</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>장지은</t>
+          <t>이성원</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>010-7141-6474</t>
+          <t>010-4188-2847</t>
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
@@ -1274,12 +1274,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>GG-A-26-001</t>
+          <t>GG-A-26-002</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>(주) 대한솔루션</t>
+          <t>주식회사 대솔오시스</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1289,22 +1289,22 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>1398100699</t>
+          <t>1398115533</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>권회현, 오문석, 권충호</t>
+          <t>권민호</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>윤종혁</t>
+          <t>장지은</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>010-9252-5623</t>
+          <t>010-7141-6474</t>
         </is>
       </c>
       <c r="H22" s="2" t="n">
@@ -1329,12 +1329,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-006</t>
+          <t>GG-A-26-001</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>(주)오성기전</t>
+          <t>(주) 대한솔루션</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1344,22 +1344,22 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>1318629038</t>
+          <t>1398100699</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>장순보</t>
+          <t>권회현, 오문석, 권충호</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>이미래</t>
+          <t>윤종혁</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>010-2513-4454</t>
+          <t>010-9252-5623</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
@@ -1384,41 +1384,41 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-005</t>
+          <t>GG-M-26-006</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>(주)윤성에프앤씨</t>
+          <t>(주)오성기전</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>경기도 안성시</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>1348150350</t>
+          <t>1318629038</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>박치영</t>
+          <t>장순보</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>윤성현</t>
+          <t>이미래</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>010-9914-7989</t>
+          <t>010-2513-4454</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>288.0</v>
+        <v>80.0</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -1439,41 +1439,41 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-004</t>
+          <t>GG-M-26-005</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>(주)백콤</t>
+          <t>(주)윤성에프앤씨</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 안성시</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>1308628716</t>
+          <t>1348150350</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>이석원</t>
+          <t>박치영</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>서범석</t>
+          <t>윤성현</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>010-5055-4994</t>
+          <t>010-9914-7989</t>
         </is>
       </c>
       <c r="H25" s="2" t="n">
-        <v>47.0</v>
+        <v>288.0</v>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
@@ -1482,53 +1482,53 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-003</t>
+          <t>GG-M-26-004</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>한국미쓰비시엘리베이터(주)</t>
+          <t>(주)백콤</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 연수구</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>1378514007</t>
+          <t>1308628716</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>김성빈</t>
+          <t>이석원</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>장연욱</t>
+          <t>서범석</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>010-3976-0627</t>
+          <t>010-5055-4994</t>
         </is>
       </c>
       <c r="H26" s="2" t="n">
-        <v>209.0</v>
+        <v>47.0</v>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
@@ -1549,92 +1549,92 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>GG-S-26-002</t>
+          <t>GG-M-26-003</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>주식회사 웨이투웨이</t>
+          <t>한국미쓰비시엘리베이터(주)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>경기 시흥시</t>
+          <t>인천광역시 연수구</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>1408181673</t>
+          <t>1378514007</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>민금기</t>
+          <t>김성빈</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>김미선</t>
+          <t>장연욱</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>010-9301-4564</t>
+          <t>010-3976-0627</t>
         </is>
       </c>
       <c r="H27" s="2" t="n">
-        <v>0.0</v>
+        <v>209.0</v>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>비활성</t>
+          <t>정상</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>최승혜</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-002</t>
+          <t>GG-S-26-002</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>비카코리아 주식회사</t>
+          <t>주식회사 웨이투웨이</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>경기도 오산시</t>
+          <t>경기 시흥시</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>6108128707</t>
+          <t>1408181673</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>이덕우</t>
+          <t>민금기</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>이진형</t>
+          <t>김미선</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>010-4026-3019</t>
+          <t>010-9301-4564</t>
         </is>
       </c>
       <c r="H28" s="2" t="n">
@@ -1642,58 +1642,58 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>정상</t>
+          <t>비활성</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>최승혜</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>CN-E-26-001</t>
+          <t>GG-M-26-002</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>(주)디바이스</t>
+          <t>비카코리아 주식회사</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>충청남도 천안시 서북구</t>
+          <t>경기도 오산시</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>3128157991</t>
+          <t>6108128707</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>최봉진, 방인호</t>
+          <t>이덕우</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>김용호</t>
+          <t>이진형</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>010-3474-3716</t>
+          <t>010-4026-3019</t>
         </is>
       </c>
       <c r="H29" s="2" t="n">
-        <v>70.0</v>
+        <v>157.0</v>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
@@ -1714,41 +1714,41 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-003</t>
+          <t>CN-E-26-001</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>(주)지에프에스</t>
+          <t>(주)디바이스</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>경기도 의정부시</t>
+          <t>충청남도 천안시 서북구</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>1278107419</t>
+          <t>3128157991</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>김태호,김현식</t>
+          <t>최봉진, 방인호</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>임승현</t>
+          <t>김용호</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>010-9516-5508</t>
+          <t>010-3474-3716</t>
         </is>
       </c>
       <c r="H30" s="2" t="n">
-        <v>0.0</v>
+        <v>70.0</v>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
@@ -1757,53 +1757,53 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>김경훈</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>GB-M-26-001</t>
+          <t>GG-E-26-003</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>(주)케이피씨엠</t>
+          <t>(주)지에프에스</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>경상북도 경산시</t>
+          <t>경기도 의정부시</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>5158140973</t>
+          <t>1278107419</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>안장홍</t>
+          <t>김태호,김현식</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>이예슬</t>
+          <t>임승현</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>010-9721-4885</t>
+          <t>010-9516-5508</t>
         </is>
       </c>
       <c r="H31" s="2" t="n">
-        <v>188.0</v>
+        <v>0.0</v>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>한규범</t>
+          <t>김경훈</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -1824,41 +1824,41 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>SE-E-26-002</t>
+          <t>GB-M-26-001</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>(주)경인기술</t>
+          <t>(주)케이피씨엠</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 영등포구</t>
+          <t>경상북도 경산시</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>1138156416</t>
+          <t>5158140973</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>정진흥</t>
+          <t>안장홍</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>임성종</t>
+          <t>이예슬</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>010-2905-7307</t>
+          <t>010-9721-4885</t>
         </is>
       </c>
       <c r="H32" s="2" t="n">
-        <v>0.0</v>
+        <v>188.0</v>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
@@ -1867,49 +1867,49 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>한규범</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-002</t>
+          <t>SE-E-26-002</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>(주)코리아하이텍</t>
+          <t>(주)경인기술</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>서울특별시 영등포구</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>1348106311</t>
+          <t>1138156416</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>여승훈,오석철</t>
+          <t>정진흥</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>박진우</t>
+          <t>임성종</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>010-6377-6757</t>
+          <t>010-2905-7307</t>
         </is>
       </c>
       <c r="H33" s="2" t="n">
@@ -1934,41 +1934,41 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>SE-S-26-001</t>
+          <t>GG-E-26-002</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>에브제트아시아(주)</t>
+          <t>(주)코리아하이텍</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 강서구</t>
+          <t>경기도 안산시 단원구</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>1208731282</t>
+          <t>1348106311</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>조욱상</t>
+          <t>여승훈,오석철</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>전승헌</t>
+          <t>박진우</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>010-8833-0349</t>
+          <t>010-6377-6757</t>
         </is>
       </c>
       <c r="H34" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
@@ -1989,41 +1989,41 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-003</t>
+          <t>SE-S-26-001</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>디엔엠항공</t>
+          <t>에브제트아시아(주)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>서울특별시 강서구</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>6131783159</t>
+          <t>1208731282</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>황태부</t>
+          <t>조욱상</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>김미희</t>
+          <t>전승헌</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>010-8131-0888</t>
+          <t>010-8833-0349</t>
         </is>
       </c>
       <c r="H35" s="2" t="n">
-        <v>452.0</v>
+        <v>1.0</v>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>이정수</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -2044,41 +2044,41 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>GG-M-26-001</t>
+          <t>GN-M-26-003</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>씨트론(주)</t>
+          <t>디엔엠항공</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 계양구</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>1228159023</t>
+          <t>6131783159</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>정태화</t>
+          <t>황태부</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>양혜원</t>
+          <t>김미희</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>010-2770-7226</t>
+          <t>010-8131-0888</t>
         </is>
       </c>
       <c r="H36" s="2" t="n">
-        <v>0.0</v>
+        <v>452.0</v>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>이승건</t>
+          <t>이정수</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -2099,37 +2099,37 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>GG-B-26-001</t>
+          <t>GG-M-26-001</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>(주)알피바이오</t>
+          <t>씨트론(주)</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>경기도 화성시 만세구</t>
+          <t>인천광역시 계양구</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>7758501361</t>
+          <t>1228159023</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>윤재훈</t>
+          <t>정태화</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>노승우</t>
+          <t>양혜원</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>010-4899-3983</t>
+          <t>010-2770-7226</t>
         </is>
       </c>
       <c r="H37" s="2" t="n">
@@ -2154,41 +2154,41 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>SE-B-26-001</t>
+          <t>GG-B-26-001</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>주식회사 코젠바이오텍</t>
+          <t>(주)알피바이오</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 금천구</t>
+          <t>경기도 화성시 만세구</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>1018156320</t>
+          <t>7758501361</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>남용석, 남주현</t>
+          <t>윤재훈</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>정지만</t>
+          <t>노승우</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>010-5348-2308</t>
+          <t>010-4899-3983</t>
         </is>
       </c>
       <c r="H38" s="2" t="n">
-        <v>45.0</v>
+        <v>163.0</v>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>정경훈</t>
+          <t>이승건</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -2209,41 +2209,41 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>GG-S-26-001</t>
+          <t>SE-B-26-001</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>(주)에어로피스</t>
+          <t>주식회사 코젠바이오텍</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>서울특별시 금천구</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>1378604165</t>
+          <t>1018156320</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>송인성</t>
+          <t>남용석, 남주현</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>염요찬</t>
+          <t>정지만</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>010-8803-5930</t>
+          <t>010-5348-2308</t>
         </is>
       </c>
       <c r="H39" s="2" t="n">
-        <v>237.0</v>
+        <v>45.0</v>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>정경훈</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
@@ -2264,41 +2264,41 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>SE-M-26-006</t>
+          <t>GG-S-26-001</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>주식회사 덱스레보</t>
+          <t>(주)에어로피스</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>서울 금천구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>1198678150</t>
+          <t>1378604165</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>유재원</t>
+          <t>송인성</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>이득훈</t>
+          <t>염요찬</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>010-4119-7124</t>
+          <t>010-8803-5930</t>
         </is>
       </c>
       <c r="H40" s="2" t="n">
-        <v>10.0</v>
+        <v>237.0</v>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>정경훈</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -2319,41 +2319,41 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-002</t>
+          <t>SE-M-26-006</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>주식회사 카프마이크로</t>
+          <t>주식회사 덱스레보</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>서울 금천구</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>3148613655</t>
+          <t>1198678150</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>이인권</t>
+          <t>유재원</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>박준영</t>
+          <t>이득훈</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>010-9305-1034</t>
+          <t>010-4119-7124</t>
         </is>
       </c>
       <c r="H41" s="2" t="n">
-        <v>60.0</v>
+        <v>10.0</v>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
@@ -2362,53 +2362,53 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>이정수</t>
+          <t>정경훈</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>CN-M-26-001</t>
+          <t>GN-M-26-002</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>연합정밀(주)</t>
+          <t>주식회사 카프마이크로</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>충남 천안시 동남구</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>3128109219</t>
+          <t>3148613655</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>김은주</t>
+          <t>이인권</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>하상우</t>
+          <t>박준영</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>010-2942-3411</t>
+          <t>010-9305-1034</t>
         </is>
       </c>
       <c r="H42" s="2" t="n">
-        <v>1827.0</v>
+        <v>60.0</v>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>이정수</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -2429,41 +2429,41 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>SE-E-26-001</t>
+          <t>CN-M-26-001</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>(주)우리기술</t>
+          <t>연합정밀(주)</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>서울 마포구</t>
+          <t>충남 천안시 동남구</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>1128138619</t>
+          <t>3128109219</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>노갑선</t>
+          <t>김은주</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>이원근</t>
+          <t>하상우</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>010-9792-8173</t>
+          <t>010-2942-3411</t>
         </is>
       </c>
       <c r="H43" s="2" t="n">
-        <v>84.0</v>
+        <v>1827.0</v>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
@@ -2472,53 +2472,53 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>GN-M-26-001</t>
+          <t>SE-E-26-001</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>(주)신화프리텍</t>
+          <t>(주)우리기술</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>경남 창원시 성산구</t>
+          <t>서울 마포구</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>6088151660</t>
+          <t>1128138619</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>배진기</t>
+          <t>노갑선</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>최문정</t>
+          <t>이원근</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>010-8669-1533</t>
+          <t>010-9792-8173</t>
         </is>
       </c>
       <c r="H44" s="2" t="n">
-        <v>1070.0</v>
+        <v>84.0</v>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>송민규</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -2539,41 +2539,41 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>CB-A-26-001</t>
+          <t>GN-M-26-001</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>(주)한국기능공사</t>
+          <t>(주)신화프리텍</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>충북 음성군</t>
+          <t>경남 창원시 성산구</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>1258112293</t>
+          <t>6088151660</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>김성국, 김성만</t>
+          <t>배진기</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>하갑봉</t>
+          <t>최문정</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>010-5655-3719</t>
+          <t>010-8669-1533</t>
         </is>
       </c>
       <c r="H45" s="2" t="n">
-        <v>614.0</v>
+        <v>1183.0</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>송민규</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -2594,41 +2594,41 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>GG-E-26-001</t>
+          <t>CB-A-26-001</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>(주)휴니드테크놀러지스</t>
+          <t>(주)한국기능공사</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>인천 연수구</t>
+          <t>충북 음성군</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>1238106174</t>
+          <t>1258112293</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>이철승(공동대표),김영호(공동대표)</t>
+          <t>김성국, 김성만</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>신원범</t>
+          <t>하갑봉</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>010-8543-4717</t>
+          <t>010-5655-3719</t>
         </is>
       </c>
       <c r="H46" s="2" t="n">
-        <v>916.0</v>
+        <v>614.0</v>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
@@ -2637,53 +2637,53 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>정상훈</t>
+          <t>전원준</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>CN-A-26-001</t>
+          <t>GG-E-26-001</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>(주)서연이화 아산공장</t>
+          <t>(주)휴니드테크놀러지스</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>충남 아산시</t>
+          <t>인천 연수구</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>3128564374</t>
+          <t>1238106174</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>강용석</t>
+          <t>이철승(공동대표),김영호(공동대표)</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>류제형</t>
+          <t>신원범</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>010-8210-1082</t>
+          <t>010-8543-4717</t>
         </is>
       </c>
       <c r="H47" s="2" t="n">
-        <v>84.0</v>
+        <v>916.0</v>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>전원준</t>
+          <t>정상훈</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -2704,53 +2704,108 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
+          <t>CN-A-26-001</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>(주)서연이화 아산공장</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>충남 아산시</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>3128564374</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>강용석</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>류제형</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>010-8210-1082</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>85.0</v>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>정상</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>전원준</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
           <t>SE-M-26-005</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>코리아인스트루먼트(주)</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>서울 구로구</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>1018145861</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>최선구</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>KIC관리자</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>010-0000-0000</t>
         </is>
       </c>
-      <c r="H48" s="2" t="n">
+      <c r="H49" s="2" t="n">
         <v>0.0</v>
       </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr">
         <is>
           <t>비활성</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="J49" s="2" t="inlineStr">
         <is>
           <t>KIC관리자</t>
         </is>
       </c>
-      <c r="K48" s="2" t="inlineStr">
+      <c r="K49" s="2" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>

</xml_diff>